<commit_message>
Actualización BD participantes; ignore temp Excel files
</commit_message>
<xml_diff>
--- a/BD participantes.xlsx
+++ b/BD participantes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/upmsj/Desktop/UPMSJ /JF/polla/app/pm_project jun/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B258C627-4CCE-BC4C-B8FF-1EB0AC41B76F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8EA1D6E-2C38-9F45-B171-F183B2311D17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28800" yWindow="2560" windowWidth="28800" windowHeight="17400" xr2:uid="{FA559016-7FAB-0B47-8ABB-CBD3A3CB183F}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="127">
   <si>
     <t>ID</t>
   </si>
@@ -411,6 +411,12 @@
   </si>
   <si>
     <t>J29QPX</t>
+  </si>
+  <si>
+    <t>8PV3KZ</t>
+  </si>
+  <si>
+    <t>Jeffry Trujillo</t>
   </si>
 </sst>
 </file>
@@ -476,8 +482,8 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -837,7 +843,7 @@
       <c r="A2" s="2">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="2" t="s">
         <v>93</v>
       </c>
       <c r="C2" s="3" t="s">
@@ -848,7 +854,7 @@
       <c r="A3" s="2">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="2" t="s">
         <v>63</v>
       </c>
       <c r="C3" s="3" t="s">
@@ -859,7 +865,7 @@
       <c r="A4" s="2">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="2" t="s">
         <v>64</v>
       </c>
       <c r="C4" s="3" t="s">
@@ -870,7 +876,7 @@
       <c r="A5" s="2">
         <v>4</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="2" t="s">
         <v>65</v>
       </c>
       <c r="C5" s="3" t="s">
@@ -881,7 +887,7 @@
       <c r="A6" s="2">
         <v>5</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="2" t="s">
         <v>66</v>
       </c>
       <c r="C6" s="3" t="s">
@@ -892,7 +898,7 @@
       <c r="A7" s="2">
         <v>6</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="2" t="s">
         <v>80</v>
       </c>
       <c r="C7" s="3" t="s">
@@ -903,7 +909,7 @@
       <c r="A8" s="2">
         <v>7</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="2" t="s">
         <v>95</v>
       </c>
       <c r="C8" s="3" t="s">
@@ -914,7 +920,7 @@
       <c r="A9" s="2">
         <v>8</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="2" t="s">
         <v>96</v>
       </c>
       <c r="C9" s="3" t="s">
@@ -925,7 +931,7 @@
       <c r="A10" s="2">
         <v>9</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="2" t="s">
         <v>67</v>
       </c>
       <c r="C10" s="3" t="s">
@@ -936,7 +942,7 @@
       <c r="A11" s="2">
         <v>10</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="2" t="s">
         <v>68</v>
       </c>
       <c r="C11" s="3" t="s">
@@ -947,7 +953,7 @@
       <c r="A12" s="2">
         <v>11</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="2" t="s">
         <v>69</v>
       </c>
       <c r="C12" s="3" t="s">
@@ -958,7 +964,7 @@
       <c r="A13" s="2">
         <v>12</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="2" t="s">
         <v>70</v>
       </c>
       <c r="C13" s="3" t="s">
@@ -969,7 +975,7 @@
       <c r="A14" s="2">
         <v>13</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="2" t="s">
         <v>71</v>
       </c>
       <c r="C14" s="3" t="s">
@@ -980,7 +986,7 @@
       <c r="A15" s="2">
         <v>14</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="2" t="s">
         <v>72</v>
       </c>
       <c r="C15" s="3" t="s">
@@ -991,7 +997,7 @@
       <c r="A16" s="2">
         <v>15</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="2" t="s">
         <v>73</v>
       </c>
       <c r="C16" s="3" t="s">
@@ -1002,7 +1008,7 @@
       <c r="A17" s="2">
         <v>16</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="2" t="s">
         <v>94</v>
       </c>
       <c r="C17" s="3" t="s">
@@ -1013,7 +1019,7 @@
       <c r="A18" s="2">
         <v>17</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="2" t="s">
         <v>74</v>
       </c>
       <c r="C18" s="3" t="s">
@@ -1024,7 +1030,7 @@
       <c r="A19" s="2">
         <v>18</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="2" t="s">
         <v>75</v>
       </c>
       <c r="C19" s="3" t="s">
@@ -1035,7 +1041,7 @@
       <c r="A20" s="2">
         <v>19</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="2" t="s">
         <v>76</v>
       </c>
       <c r="C20" s="3" t="s">
@@ -1046,7 +1052,7 @@
       <c r="A21" s="2">
         <v>20</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="2" t="s">
         <v>77</v>
       </c>
       <c r="C21" s="3" t="s">
@@ -1057,7 +1063,7 @@
       <c r="A22" s="2">
         <v>21</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="2" t="s">
         <v>78</v>
       </c>
       <c r="C22" s="3" t="s">
@@ -1068,7 +1074,7 @@
       <c r="A23" s="2">
         <v>22</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="B23" s="2" t="s">
         <v>79</v>
       </c>
       <c r="C23" s="3" t="s">
@@ -1079,7 +1085,7 @@
       <c r="A24" s="2">
         <v>23</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B24" s="2" t="s">
         <v>81</v>
       </c>
       <c r="C24" s="3" t="s">
@@ -1090,7 +1096,7 @@
       <c r="A25" s="2">
         <v>24</v>
       </c>
-      <c r="B25" s="4" t="s">
+      <c r="B25" s="2" t="s">
         <v>82</v>
       </c>
       <c r="C25" s="3" t="s">
@@ -1101,7 +1107,7 @@
       <c r="A26" s="2">
         <v>25</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="B26" s="2" t="s">
         <v>83</v>
       </c>
       <c r="C26" s="3" t="s">
@@ -1112,7 +1118,7 @@
       <c r="A27" s="2">
         <v>26</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="B27" s="2" t="s">
         <v>84</v>
       </c>
       <c r="C27" s="3" t="s">
@@ -1123,7 +1129,7 @@
       <c r="A28" s="2">
         <v>27</v>
       </c>
-      <c r="B28" s="4" t="s">
+      <c r="B28" s="2" t="s">
         <v>85</v>
       </c>
       <c r="C28" s="3" t="s">
@@ -1134,7 +1140,7 @@
       <c r="A29" s="2">
         <v>28</v>
       </c>
-      <c r="B29" s="4" t="s">
+      <c r="B29" s="2" t="s">
         <v>86</v>
       </c>
       <c r="C29" s="3" t="s">
@@ -1145,7 +1151,7 @@
       <c r="A30" s="2">
         <v>29</v>
       </c>
-      <c r="B30" s="4" t="s">
+      <c r="B30" s="2" t="s">
         <v>87</v>
       </c>
       <c r="C30" s="3" t="s">
@@ -1156,7 +1162,7 @@
       <c r="A31" s="2">
         <v>30</v>
       </c>
-      <c r="B31" s="4" t="s">
+      <c r="B31" s="2" t="s">
         <v>88</v>
       </c>
       <c r="C31" s="3" t="s">
@@ -1167,7 +1173,7 @@
       <c r="A32" s="2">
         <v>31</v>
       </c>
-      <c r="B32" s="4" t="s">
+      <c r="B32" s="2" t="s">
         <v>89</v>
       </c>
       <c r="C32" s="3" t="s">
@@ -1178,7 +1184,7 @@
       <c r="A33" s="2">
         <v>32</v>
       </c>
-      <c r="B33" s="4" t="s">
+      <c r="B33" s="2" t="s">
         <v>90</v>
       </c>
       <c r="C33" s="3" t="s">
@@ -1189,7 +1195,7 @@
       <c r="A34" s="2">
         <v>33</v>
       </c>
-      <c r="B34" s="4" t="s">
+      <c r="B34" s="2" t="s">
         <v>91</v>
       </c>
       <c r="C34" s="3" t="s">
@@ -1200,7 +1206,7 @@
       <c r="A35" s="2">
         <v>34</v>
       </c>
-      <c r="B35" s="4" t="s">
+      <c r="B35" s="2" t="s">
         <v>92</v>
       </c>
       <c r="C35" s="3" t="s">
@@ -1211,7 +1217,7 @@
       <c r="A36" s="2">
         <v>35</v>
       </c>
-      <c r="B36" s="4" t="s">
+      <c r="B36" s="2" t="s">
         <v>97</v>
       </c>
       <c r="C36" s="3" t="s">
@@ -1222,7 +1228,7 @@
       <c r="A37" s="2">
         <v>36</v>
       </c>
-      <c r="B37" s="4" t="s">
+      <c r="B37" s="2" t="s">
         <v>98</v>
       </c>
       <c r="C37" s="3" t="s">
@@ -1233,7 +1239,7 @@
       <c r="A38" s="2">
         <v>37</v>
       </c>
-      <c r="B38" s="4" t="s">
+      <c r="B38" s="2" t="s">
         <v>99</v>
       </c>
       <c r="C38" s="3" t="s">
@@ -1244,7 +1250,7 @@
       <c r="A39" s="2">
         <v>38</v>
       </c>
-      <c r="B39" s="4" t="s">
+      <c r="B39" s="2" t="s">
         <v>100</v>
       </c>
       <c r="C39" s="3" t="s">
@@ -1255,7 +1261,7 @@
       <c r="A40" s="2">
         <v>39</v>
       </c>
-      <c r="B40" s="4" t="s">
+      <c r="B40" s="2" t="s">
         <v>101</v>
       </c>
       <c r="C40" s="3" t="s">
@@ -1266,7 +1272,7 @@
       <c r="A41" s="2">
         <v>40</v>
       </c>
-      <c r="B41" s="4" t="s">
+      <c r="B41" s="2" t="s">
         <v>102</v>
       </c>
       <c r="C41" s="3" t="s">
@@ -1277,7 +1283,7 @@
       <c r="A42" s="2">
         <v>41</v>
       </c>
-      <c r="B42" s="4" t="s">
+      <c r="B42" s="2" t="s">
         <v>103</v>
       </c>
       <c r="C42" s="3" t="s">
@@ -1288,7 +1294,7 @@
       <c r="A43" s="2">
         <v>42</v>
       </c>
-      <c r="B43" s="4" t="s">
+      <c r="B43" s="2" t="s">
         <v>104</v>
       </c>
       <c r="C43" s="3" t="s">
@@ -1299,7 +1305,7 @@
       <c r="A44" s="2">
         <v>43</v>
       </c>
-      <c r="B44" s="4" t="s">
+      <c r="B44" s="2" t="s">
         <v>105</v>
       </c>
       <c r="C44" s="3" t="s">
@@ -1310,7 +1316,7 @@
       <c r="A45" s="2">
         <v>44</v>
       </c>
-      <c r="B45" s="4" t="s">
+      <c r="B45" s="2" t="s">
         <v>106</v>
       </c>
       <c r="C45" s="3" t="s">
@@ -1321,7 +1327,7 @@
       <c r="A46" s="2">
         <v>45</v>
       </c>
-      <c r="B46" s="4" t="s">
+      <c r="B46" s="2" t="s">
         <v>118</v>
       </c>
       <c r="C46" s="3" t="s">
@@ -1332,7 +1338,7 @@
       <c r="A47" s="2">
         <v>46</v>
       </c>
-      <c r="B47" s="4" t="s">
+      <c r="B47" s="2" t="s">
         <v>119</v>
       </c>
       <c r="C47" s="3" t="s">
@@ -1343,7 +1349,7 @@
       <c r="A48" s="2">
         <v>47</v>
       </c>
-      <c r="B48" s="4" t="s">
+      <c r="B48" s="2" t="s">
         <v>120</v>
       </c>
       <c r="C48" s="3" t="s">
@@ -1354,7 +1360,7 @@
       <c r="A49" s="2">
         <v>48</v>
       </c>
-      <c r="B49" s="4" t="s">
+      <c r="B49" s="2" t="s">
         <v>121</v>
       </c>
       <c r="C49" s="3" t="s">
@@ -1365,7 +1371,7 @@
       <c r="A50" s="2">
         <v>49</v>
       </c>
-      <c r="B50" s="4" t="s">
+      <c r="B50" s="2" t="s">
         <v>122</v>
       </c>
       <c r="C50" s="3" t="s">
@@ -1376,7 +1382,7 @@
       <c r="A51" s="2">
         <v>50</v>
       </c>
-      <c r="B51" s="4" t="s">
+      <c r="B51" s="2" t="s">
         <v>115</v>
       </c>
       <c r="C51" s="3" t="s">
@@ -1387,7 +1393,7 @@
       <c r="A52" s="2">
         <v>51</v>
       </c>
-      <c r="B52" s="4" t="s">
+      <c r="B52" s="2" t="s">
         <v>107</v>
       </c>
       <c r="C52" s="3" t="s">
@@ -1398,7 +1404,7 @@
       <c r="A53" s="2">
         <v>52</v>
       </c>
-      <c r="B53" s="4" t="s">
+      <c r="B53" s="2" t="s">
         <v>109</v>
       </c>
       <c r="C53" s="3" t="s">
@@ -1409,7 +1415,7 @@
       <c r="A54" s="2">
         <v>53</v>
       </c>
-      <c r="B54" s="4" t="s">
+      <c r="B54" s="2" t="s">
         <v>108</v>
       </c>
       <c r="C54" s="3" t="s">
@@ -1420,7 +1426,7 @@
       <c r="A55" s="2">
         <v>54</v>
       </c>
-      <c r="B55" s="4" t="s">
+      <c r="B55" s="2" t="s">
         <v>110</v>
       </c>
       <c r="C55" s="3" t="s">
@@ -1431,7 +1437,7 @@
       <c r="A56" s="2">
         <v>55</v>
       </c>
-      <c r="B56" s="4" t="s">
+      <c r="B56" s="2" t="s">
         <v>117</v>
       </c>
       <c r="C56" s="3" t="s">
@@ -1442,7 +1448,7 @@
       <c r="A57" s="2">
         <v>56</v>
       </c>
-      <c r="B57" s="4" t="s">
+      <c r="B57" s="2" t="s">
         <v>111</v>
       </c>
       <c r="C57" s="3" t="s">
@@ -1453,7 +1459,7 @@
       <c r="A58" s="2">
         <v>57</v>
       </c>
-      <c r="B58" s="4" t="s">
+      <c r="B58" s="2" t="s">
         <v>112</v>
       </c>
       <c r="C58" s="3" t="s">
@@ -1464,7 +1470,7 @@
       <c r="A59" s="2">
         <v>58</v>
       </c>
-      <c r="B59" s="4" t="s">
+      <c r="B59" s="2" t="s">
         <v>113</v>
       </c>
       <c r="C59" s="3" t="s">
@@ -1475,7 +1481,7 @@
       <c r="A60" s="2">
         <v>59</v>
       </c>
-      <c r="B60" s="4" t="s">
+      <c r="B60" s="2" t="s">
         <v>114</v>
       </c>
       <c r="C60" s="3" t="s">
@@ -1486,7 +1492,7 @@
       <c r="A61" s="2">
         <v>60</v>
       </c>
-      <c r="B61" s="4" t="s">
+      <c r="B61" s="2" t="s">
         <v>116</v>
       </c>
       <c r="C61" s="3" t="s">
@@ -1497,11 +1503,22 @@
       <c r="A62" s="2">
         <v>61</v>
       </c>
-      <c r="B62" s="4" t="s">
+      <c r="B62" s="2" t="s">
         <v>123</v>
       </c>
       <c r="C62" s="2" t="s">
         <v>124</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A63" s="2">
+        <v>62</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="C63" s="4" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Texto T. Extra/Penales; avatar 200px calidad 0.85
</commit_message>
<xml_diff>
--- a/BD participantes.xlsx
+++ b/BD participantes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/upmsj/Desktop/UPMSJ /JF/polla/app/pm_project jun/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8EA1D6E-2C38-9F45-B171-F183B2311D17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7061657-37CC-AC45-BF3D-98EA9B9FD8DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28800" yWindow="2560" windowWidth="28800" windowHeight="17400" xr2:uid="{FA559016-7FAB-0B47-8ABB-CBD3A3CB183F}"/>
+    <workbookView xWindow="4940" yWindow="2920" windowWidth="28800" windowHeight="17400" xr2:uid="{FA559016-7FAB-0B47-8ABB-CBD3A3CB183F}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="133">
   <si>
     <t>ID</t>
   </si>
@@ -275,12 +275,6 @@
     <t>Benja Mucarsel B</t>
   </si>
   <si>
-    <t>Oscar Arteaga</t>
-  </si>
-  <si>
-    <t>Sebastian Larco</t>
-  </si>
-  <si>
     <t>Hipa Vásquez</t>
   </si>
   <si>
@@ -347,9 +341,6 @@
     <t>Luis Moreno</t>
   </si>
   <si>
-    <t>Jose Viera</t>
-  </si>
-  <si>
     <t>Paco Ortiz</t>
   </si>
   <si>
@@ -362,9 +353,6 @@
     <t>Carlos Castro</t>
   </si>
   <si>
-    <t>Carlitos y Patty</t>
-  </si>
-  <si>
     <t>Doménica Larrea</t>
   </si>
   <si>
@@ -417,6 +405,36 @@
   </si>
   <si>
     <t>Jeffry Trujillo</t>
+  </si>
+  <si>
+    <t>Fabián Procel</t>
+  </si>
+  <si>
+    <t>UHOAFN</t>
+  </si>
+  <si>
+    <t>Jonathan Vásquez</t>
+  </si>
+  <si>
+    <t>G9DBE7</t>
+  </si>
+  <si>
+    <t>Carlos F Castro</t>
+  </si>
+  <si>
+    <t>Sebastián Larco</t>
+  </si>
+  <si>
+    <t>Óscar Arteaga</t>
+  </si>
+  <si>
+    <t>José Viera</t>
+  </si>
+  <si>
+    <t>Kevin Puga</t>
+  </si>
+  <si>
+    <t>DX9TWC</t>
   </si>
 </sst>
 </file>
@@ -844,7 +862,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>3</v>
@@ -899,7 +917,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>80</v>
+        <v>128</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>8</v>
@@ -910,7 +928,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>9</v>
@@ -921,7 +939,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>10</v>
@@ -1009,7 +1027,7 @@
         <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>18</v>
@@ -1075,7 +1093,7 @@
         <v>22</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>79</v>
+        <v>129</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>24</v>
@@ -1086,7 +1104,7 @@
         <v>23</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>25</v>
@@ -1097,7 +1115,7 @@
         <v>24</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>26</v>
@@ -1108,7 +1126,7 @@
         <v>25</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>27</v>
@@ -1119,7 +1137,7 @@
         <v>26</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C27" s="3" t="s">
         <v>28</v>
@@ -1130,7 +1148,7 @@
         <v>27</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>29</v>
@@ -1141,7 +1159,7 @@
         <v>28</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C29" s="3" t="s">
         <v>30</v>
@@ -1152,7 +1170,7 @@
         <v>29</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>31</v>
@@ -1163,7 +1181,7 @@
         <v>30</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C31" s="3" t="s">
         <v>32</v>
@@ -1174,7 +1192,7 @@
         <v>31</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C32" s="3" t="s">
         <v>33</v>
@@ -1185,7 +1203,7 @@
         <v>32</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C33" s="3" t="s">
         <v>34</v>
@@ -1196,7 +1214,7 @@
         <v>33</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C34" s="3" t="s">
         <v>35</v>
@@ -1207,7 +1225,7 @@
         <v>34</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C35" s="3" t="s">
         <v>36</v>
@@ -1218,7 +1236,7 @@
         <v>35</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C36" s="3" t="s">
         <v>37</v>
@@ -1229,7 +1247,7 @@
         <v>36</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C37" s="3" t="s">
         <v>38</v>
@@ -1240,7 +1258,7 @@
         <v>37</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C38" s="3" t="s">
         <v>39</v>
@@ -1251,7 +1269,7 @@
         <v>38</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C39" s="3" t="s">
         <v>40</v>
@@ -1262,7 +1280,7 @@
         <v>39</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C40" s="3" t="s">
         <v>41</v>
@@ -1273,7 +1291,7 @@
         <v>40</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C41" s="3" t="s">
         <v>42</v>
@@ -1284,7 +1302,7 @@
         <v>41</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>103</v>
+        <v>130</v>
       </c>
       <c r="C42" s="3" t="s">
         <v>43</v>
@@ -1295,7 +1313,7 @@
         <v>42</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C43" s="3" t="s">
         <v>44</v>
@@ -1306,7 +1324,7 @@
         <v>43</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C44" s="3" t="s">
         <v>45</v>
@@ -1317,7 +1335,7 @@
         <v>44</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C45" s="3" t="s">
         <v>46</v>
@@ -1328,7 +1346,7 @@
         <v>45</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="C46" s="3" t="s">
         <v>47</v>
@@ -1339,7 +1357,7 @@
         <v>46</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="C47" s="3" t="s">
         <v>48</v>
@@ -1350,7 +1368,7 @@
         <v>47</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="C48" s="3" t="s">
         <v>49</v>
@@ -1361,7 +1379,7 @@
         <v>48</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="C49" s="3" t="s">
         <v>50</v>
@@ -1372,7 +1390,7 @@
         <v>49</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="C50" s="3" t="s">
         <v>51</v>
@@ -1383,7 +1401,7 @@
         <v>50</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="C51" s="3" t="s">
         <v>52</v>
@@ -1394,7 +1412,7 @@
         <v>51</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C52" s="3" t="s">
         <v>53</v>
@@ -1405,7 +1423,7 @@
         <v>52</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="C53" s="3" t="s">
         <v>54</v>
@@ -1416,7 +1434,7 @@
         <v>53</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>108</v>
+        <v>127</v>
       </c>
       <c r="C54" s="3" t="s">
         <v>55</v>
@@ -1427,7 +1445,7 @@
         <v>54</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="C55" s="3" t="s">
         <v>56</v>
@@ -1438,7 +1456,7 @@
         <v>55</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="C56" s="3" t="s">
         <v>57</v>
@@ -1449,7 +1467,7 @@
         <v>56</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="C57" s="3" t="s">
         <v>58</v>
@@ -1460,7 +1478,7 @@
         <v>57</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="C58" s="3" t="s">
         <v>59</v>
@@ -1471,7 +1489,7 @@
         <v>58</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="C59" s="3" t="s">
         <v>60</v>
@@ -1482,7 +1500,7 @@
         <v>59</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="C60" s="3" t="s">
         <v>61</v>
@@ -1493,7 +1511,7 @@
         <v>60</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="C61" s="3" t="s">
         <v>62</v>
@@ -1504,10 +1522,10 @@
         <v>61</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.2">
@@ -1515,43 +1533,70 @@
         <v>62</v>
       </c>
       <c r="B63" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="C63" s="4" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A64" s="2">
+        <v>63</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="D64" s="2"/>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A65" s="2">
+        <v>64</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="C65" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="C63" s="4" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="D64" s="2"/>
-    </row>
-    <row r="65" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D65" s="2"/>
     </row>
-    <row r="66" spans="4:4" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A66" s="2">
+        <v>65</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>132</v>
+      </c>
       <c r="D66" s="2"/>
     </row>
-    <row r="67" spans="4:4" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
       <c r="D67" s="2"/>
     </row>
-    <row r="68" spans="4:4" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
       <c r="D68" s="2"/>
     </row>
-    <row r="69" spans="4:4" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
       <c r="D69" s="2"/>
     </row>
-    <row r="70" spans="4:4" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
       <c r="D70" s="2"/>
     </row>
-    <row r="71" spans="4:4" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.2">
       <c r="D71" s="2"/>
     </row>
-    <row r="72" spans="4:4" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.2">
       <c r="D72" s="2"/>
     </row>
-    <row r="73" spans="4:4" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
       <c r="D73" s="2"/>
     </row>
-    <row r="74" spans="4:4" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
       <c r="D74" s="2"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
admin editor: partidos futuro/hoY primero, pasados al final
</commit_message>
<xml_diff>
--- a/BD participantes.xlsx
+++ b/BD participantes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/upmsj/Desktop/UPMSJ /JF/polla/app/pm_project jun/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E13F5F92-0B25-6840-945F-A7CD8D013485}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3878CD40-6F92-FB41-91C2-A5E5E94C3D0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28800" yWindow="2560" windowWidth="28800" windowHeight="17400" xr2:uid="{FA559016-7FAB-0B47-8ABB-CBD3A3CB183F}"/>
   </bookViews>
@@ -386,9 +386,6 @@
     <t>Roberto Peñafiel</t>
   </si>
   <si>
-    <t>Hernán Espinosa</t>
-  </si>
-  <si>
     <t>J29QPX</t>
   </si>
   <si>
@@ -435,6 +432,9 @@
   </si>
   <si>
     <t>Oscar Arteaga</t>
+  </si>
+  <si>
+    <t>Hernán Espinoza</t>
   </si>
 </sst>
 </file>
@@ -917,7 +917,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>8</v>
@@ -939,7 +939,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>10</v>
@@ -961,7 +961,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>12</v>
@@ -1093,7 +1093,7 @@
         <v>22</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>24</v>
@@ -1214,7 +1214,7 @@
         <v>33</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C34" s="3" t="s">
         <v>35</v>
@@ -1302,7 +1302,7 @@
         <v>41</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C42" s="3" t="s">
         <v>43</v>
@@ -1434,7 +1434,7 @@
         <v>53</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C54" s="3" t="s">
         <v>55</v>
@@ -1522,10 +1522,10 @@
         <v>61</v>
       </c>
       <c r="B62" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="C62" s="2" t="s">
         <v>116</v>
-      </c>
-      <c r="C62" s="2" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.2">
@@ -1533,10 +1533,10 @@
         <v>62</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C63" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.2">
@@ -1544,10 +1544,10 @@
         <v>63</v>
       </c>
       <c r="B64" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="C64" s="2" t="s">
         <v>120</v>
-      </c>
-      <c r="C64" s="2" t="s">
-        <v>121</v>
       </c>
       <c r="D64" s="2"/>
     </row>
@@ -1556,10 +1556,10 @@
         <v>64</v>
       </c>
       <c r="B65" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C65" s="2" t="s">
         <v>122</v>
-      </c>
-      <c r="C65" s="2" t="s">
-        <v>123</v>
       </c>
       <c r="D65" s="2"/>
     </row>
@@ -1568,10 +1568,10 @@
         <v>65</v>
       </c>
       <c r="B66" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="C66" s="2" t="s">
         <v>127</v>
-      </c>
-      <c r="C66" s="2" t="s">
-        <v>128</v>
       </c>
       <c r="D66" s="2"/>
     </row>

</xml_diff>